<commit_message>
Criacao de nova classe savi para representar a pagina web, alteracao nos tipos atributos de planilha, criação de novos metodos para clicar e escrever em campos via selenium e alteracao na classe automacao para utilizar majoritariamente selenium envez de robot.
</commit_message>
<xml_diff>
--- a/Planilha modelo.xlsx
+++ b/Planilha modelo.xlsx
@@ -2,6 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
+  <bookViews>
+    <workbookView activeTab="0"/>
+  </bookViews>
   <sheets>
     <sheet state="visible" name="Folha1" sheetId="1" r:id="rId4"/>
   </sheets>
@@ -13,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1122" uniqueCount="56">
   <si>
     <t>senha</t>
   </si>
@@ -169,6 +172,18 @@
   </si>
   <si>
     <t>D</t>
+  </si>
+  <si>
+    <t>Honorário Médico processado com sucesso.</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Número de guia já utilizado para outro honorário.</t>
+  </si>
+  <si>
+    <t>ERRO</t>
   </si>
 </sst>
 </file>
@@ -542,22 +557,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
+  <dimension ref="A1:AC995"/>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="10.25"/>
-    <col customWidth="1" min="2" max="2" width="13.0"/>
-    <col customWidth="1" min="3" max="3" width="10.63"/>
-    <col customWidth="1" min="4" max="4" width="10.13"/>
-    <col customWidth="1" min="5" max="5" width="7.25"/>
-    <col customWidth="1" min="6" max="6" width="11.5"/>
-    <col customWidth="1" min="7" max="7" width="12.38"/>
-    <col customWidth="1" min="8" max="8" width="19.88"/>
-    <col customWidth="1" min="9" max="9" width="17.0"/>
-    <col customWidth="1" min="10" max="10" width="8.75"/>
-    <col customWidth="1" min="11" max="12" width="10.5"/>
-    <col customWidth="1" min="13" max="13" width="4.13"/>
-    <col customWidth="1" min="14" max="14" width="6.63"/>
-    <col customWidth="1" min="15" max="15" width="12.75"/>
+    <col min="1" max="1" customWidth="true" width="10.25"/>
+    <col min="2" max="2" customWidth="true" width="13.0"/>
+    <col min="3" max="3" customWidth="true" width="10.63"/>
+    <col min="4" max="4" customWidth="true" width="10.13"/>
+    <col min="5" max="5" customWidth="true" width="7.25"/>
+    <col min="6" max="6" customWidth="true" width="11.5"/>
+    <col min="7" max="7" customWidth="true" width="12.38"/>
+    <col min="8" max="8" customWidth="true" width="19.88"/>
+    <col min="9" max="9" customWidth="true" width="17.0"/>
+    <col min="10" max="10" customWidth="true" width="8.75"/>
+    <col min="11" max="12" customWidth="true" width="10.5"/>
+    <col min="13" max="13" customWidth="true" width="4.13"/>
+    <col min="14" max="14" customWidth="true" width="6.63"/>
+    <col min="15" max="15" customWidth="true" width="12.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,10 +649,10 @@
         <v>13</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="L2" s="11" t="s">
         <v>14</v>
@@ -656,6 +672,7 @@
       <c r="S2" s="12" t="s">
         <v>19</v>
       </c>
+      <c r="AC2" s="0"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
@@ -683,10 +700,10 @@
         <v>13</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="Q3" s="14">
         <v>1.0</v>
@@ -697,6 +714,7 @@
       <c r="S3" s="5" t="s">
         <v>24</v>
       </c>
+      <c r="AC3" s="0"/>
     </row>
     <row r="4">
       <c r="A4" s="15"/>
@@ -726,6 +744,7 @@
       <c r="S4" s="5" t="s">
         <v>26</v>
       </c>
+      <c r="AC4" s="0"/>
     </row>
     <row r="5">
       <c r="A5" s="15"/>

</xml_diff>

<commit_message>
Versão funcional com controllers e UI
</commit_message>
<xml_diff>
--- a/Planilha modelo.xlsx
+++ b/Planilha modelo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="57">
   <si>
     <t>senha</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>ERRO</t>
+  </si>
+  <si>
+    <t>Data Inválida. Permitido apenas atendimentos até 4 meses retroativos.</t>
   </si>
 </sst>
 </file>
@@ -700,7 +703,7 @@
         <v>13</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J3" s="5" t="s">
         <v>55</v>

</xml_diff>